<commit_message>
re-runs with correct datasets
</commit_message>
<xml_diff>
--- a/assessment/data/SC13_2025assessmentInputData_V3.xlsx
+++ b/assessment/data/SC13_2025assessmentInputData_V3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leeqi/Library/CloudStorage/GoogleDrive-leeqi@uw.edu/My Drive/SPRFMO/jjm/assessment/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32AEB7E2-A1DE-B74A-9CC6-02B350A2E1DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A345C135-246D-3B45-848A-51C1F42B6505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15120" yWindow="760" windowWidth="15120" windowHeight="18880" activeTab="3" xr2:uid="{11C67D07-EBA6-4D97-A3E6-A5FACAECFD42}"/>
+    <workbookView xWindow="15120" yWindow="760" windowWidth="15120" windowHeight="18880" activeTab="4" xr2:uid="{11C67D07-EBA6-4D97-A3E6-A5FACAECFD42}"/>
   </bookViews>
   <sheets>
     <sheet name="ageComps" sheetId="1" r:id="rId1"/>
@@ -4320,8 +4320,8 @@
         <v>1068425.3710330399</v>
       </c>
       <c r="D3" s="3">
-        <f>75+208</f>
-        <v>283</v>
+        <f>75+208000</f>
+        <v>208075</v>
       </c>
       <c r="E3" s="1">
         <v>11055.456022689201</v>
@@ -4757,12 +4757,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -4771,7 +4765,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100812D0B056278C642B7C89719D0EEC9C4" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="53e5abc0267b36fb4b4009f6291778a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f419981a-ca0a-4e56-9512-575f16b7ea2d" xmlns:ns3="5ce05999-5605-4258-98fc-62ff4522b5fb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2d299d2548571e9774994fb9c4dbbeb8" ns2:_="" ns3:_="">
     <xsd:import namespace="f419981a-ca0a-4e56-9512-575f16b7ea2d"/>
@@ -4986,16 +4980,13 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2AFB9C7-A01A-423B-A442-B6889BA2E519}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{228CE105-4287-40ED-B72B-E33A77B67D61}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -5003,7 +4994,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FFE542F3-5C46-43FB-860A-90AC96253C26}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5020,4 +5011,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2AFB9C7-A01A-423B-A442-B6889BA2E519}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>